<commit_message>
docs(inputs): correct test-case workbook descriptions
Apply the validated English wording corrections to the 40 tracked test-case workbooks while preserving seven case-specific descriptions.

All workbook hashes were verified, all files are readable, and the complete 236-test suite passes.
</commit_message>
<xml_diff>
--- a/TDD_examples/CASE_1_ITER_like_LTS/conductor_1_coupling.xlsx
+++ b/TDD_examples/CASE_1_ITER_like_LTS/conductor_1_coupling.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="contact_perimeter_flag" sheetId="1" r:id="Ra98e5c7837ac425a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="contact_perimeter" sheetId="2" r:id="Ra1bf789630f6408e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HTC_choice" sheetId="3" r:id="R901d0b1b2f4f4e4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="contact_HTC" sheetId="4" r:id="R45214fbad13241de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="thermal_contact_resistance" sheetId="5" r:id="Rab11de4d81974ff8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HTC_multiplier" sheetId="6" r:id="R53683e5eee7349d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="electric_conductance_mode" sheetId="7" r:id="R1b942f1fa6aa467f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="electric_conductance" sheetId="8" r:id="R6965f1bb46264720"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="open_perimeter_fract" sheetId="9" r:id="R735e1f67079f4690"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="interf_thickness" sheetId="10" r:id="R33ec5765cdad4b2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="trans_transp_multiplier" sheetId="11" r:id="R1f106797bae64260"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="view_factors" sheetId="12" r:id="Raf8c2bb87b0f4375"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="contact_perimeter_flag" sheetId="1" r:id="Rb3ef165e99b04401"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="contact_perimeter" sheetId="2" r:id="R6fc686984bea4a70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HTC_choice" sheetId="3" r:id="R94ab3f60c879465e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="contact_HTC" sheetId="4" r:id="R47237a8b7dc449bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="thermal_contact_resistance" sheetId="5" r:id="R59b5ecef17d74848"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HTC_multiplier" sheetId="6" r:id="Rf8134c9b4afc461d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="electric_conductance_mode" sheetId="7" r:id="Ra2614128cb674348"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="electric_conductance" sheetId="8" r:id="R5e81817ba60a48f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="open_perimeter_fract" sheetId="9" r:id="Rfa797075a2e94c85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="interf_thickness" sheetId="10" r:id="R903f16bf6aea4ee5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="trans_transp_multiplier" sheetId="11" r:id="R417f22765c6445a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="view_factors" sheetId="12" r:id="Rda77ea4c6449401a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -465,7 +465,7 @@
       <x:c r="A1" s="6"/>
       <x:c r="B1" s="6"/>
       <x:c r="C1" s="6" t="str">
-        <x:v>[m] Thickness of the interface between conductor components. For interfaces between components that are not both channels, assing in cell (comp1,comp2) the thickess of the interface of comp1  when in contact with comp2 and in cell  (comp2,comp1) the thickess of the interface of comp2  when in contact with comp1. Therefore the matrix may no longer be symmetric and also the lower triangular region should be filled.</x:v>
+        <x:v>[m] Thickness of the interface between conductor components. For interfaces between components that are not both channels, assign in cell (comp1, comp2) the thickness of the interface of comp1 when in contact with comp2, and in cell (comp2, comp1) the thickness of the interface of comp2 when in contact with comp1. Therefore, the matrix may no longer be symmetric, and the lower triangular region must also be filled.</x:v>
       </x:c>
       <x:c r="D1" s="6"/>
       <x:c r="E1" s="6"/>
@@ -1057,7 +1057,7 @@
       <x:c r="A1" s="6"/>
       <x:c r="B1" s="6"/>
       <x:c r="C1" s="6" t="str">
-        <x:v>%[] flag to define the model to compute the HTC (yellow cells are those to thake into account). flag to decide how to evaluate interface htc.</x:v>
+        <x:v>%[] Flag used to select the HTC model (yellow cells are taken into account). This flag determines how the interface HTC is evaluated.</x:v>
       </x:c>
       <x:c r="D1" s="6"/>
       <x:c r="E1" s="6"/>
@@ -1353,7 +1353,7 @@
       <x:c r="A1" s="6"/>
       <x:c r="B1" s="6"/>
       <x:c r="C1" s="6" t="str">
-        <x:v>[m2K/W] thermal contact resistance between soldi component, should be &gt;= 0; used if flag HTC_choice is 1</x:v>
+        <x:v>[m2 K/W] Thermal contact resistance between solid components; it must be &gt;= 0. Used if HTC_choice is 1.</x:v>
       </x:c>
       <x:c r="D1" s="6"/>
       <x:c r="E1" s="6"/>
@@ -1649,7 +1649,7 @@
       <x:c r="A1" s="6"/>
       <x:c r="B1" s="6"/>
       <x:c r="C1" s="6" t="str">
-        <x:v>Flag to specify the kind of electric conductance: 1 conductance per unit length (the contact is along a line as for tow cilinder); 2 = actual conductance between components.</x:v>
+        <x:v>Flag used to specify the electric conductance: 1 = conductance per unit length (the contact is along a line, as for two cylinders); 2 = actual conductance between components.</x:v>
       </x:c>
       <x:c r="D1" s="6"/>
       <x:c r="E1" s="6"/>

</xml_diff>